<commit_message>
UI Slightly polished with a better alignment and new header section
</commit_message>
<xml_diff>
--- a/VRNT_Data/admin_users.xlsx
+++ b/VRNT_Data/admin_users.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr date1904="false"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="All Users" r:id="rId3" sheetId="1"/>
+    <sheet r:id="rId1" name="All Users" sheetId="1"/>
   </sheets>
+  <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>First Name</t>
   </si>
@@ -116,52 +117,69 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3">
     <font>
-      <sz val="11.0"/>
-      <color indexed="8"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="9"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="darkGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="30"/>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0066CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="30"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="43"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="43"/>
+        <fgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left>
+        <color rgb="FF000000"/>
+      </left>
+      <right>
+        <color rgb="FF000000"/>
+      </right>
+      <top>
+        <color rgb="FF000000"/>
+      </top>
+      <bottom>
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
     <border>
       <left/>
       <right/>
@@ -170,134 +188,424 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1">
+      <alignment horizontal="general" vertical="top"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyBorder="true" applyFill="true"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4472C4"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CE22B410-AD67-4460-9B43-685B6E3E42B0}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:V2"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22.0" customWidth="true"/>
-    <col min="2" max="2" width="22.0" customWidth="true"/>
-    <col min="3" max="3" width="22.0" customWidth="true"/>
-    <col min="4" max="4" width="22.0" customWidth="true"/>
-    <col min="5" max="5" width="22.0" customWidth="true"/>
-    <col min="6" max="6" width="22.0" customWidth="true"/>
-    <col min="7" max="7" width="22.0" customWidth="true"/>
-    <col min="8" max="8" width="22.0" customWidth="true"/>
-    <col min="9" max="9" width="22.0" customWidth="true"/>
-    <col min="10" max="10" width="22.0" customWidth="true"/>
-    <col min="11" max="11" width="22.0" customWidth="true"/>
-    <col min="12" max="12" width="22.0" customWidth="true"/>
-    <col min="13" max="13" width="22.0" customWidth="true"/>
-    <col min="14" max="14" width="22.0" customWidth="true"/>
-    <col min="15" max="15" width="22.0" customWidth="true"/>
-    <col min="16" max="16" width="22.0" customWidth="true"/>
-    <col min="17" max="17" width="22.0" customWidth="true"/>
-    <col min="18" max="18" width="22.0" customWidth="true"/>
-    <col min="19" max="19" width="22.0" customWidth="true"/>
-    <col min="20" max="20" width="22.0" customWidth="true"/>
-    <col min="21" max="21" width="22.0" customWidth="true"/>
-    <col min="22" max="22" width="22.0" customWidth="true"/>
+    <col min="1" max="22" width="22.00390625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="1">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="1">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="1">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="1">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="1">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="1">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="1">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="1">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="1">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="1">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s" s="1">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s" s="1">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s" s="1">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s" s="1">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s" s="1">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s" s="1">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s" s="1">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s" s="1">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s" s="1">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s" s="1">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s" s="1">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s" s="1">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>22</v>
       </c>
@@ -366,6 +674,13 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>